<commit_message>
docs: record verified control-system run
</commit_message>
<xml_diff>
--- a/docs/Research_Project_Map.xlsx
+++ b/docs/Research_Project_Map.xlsx
@@ -2,14 +2,14 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Current Status" sheetId="1" r:id="Rcd9d83a7a03d46d9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Datasets" sheetId="2" r:id="R99e69512052a457e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Code" sheetId="3" r:id="Rf09e9ebfe6d84872"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tables" sheetId="4" r:id="Ra214646e6c5d4c19"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Figures" sheetId="5" r:id="R83df4b89d96e43ee"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Runs" sheetId="6" r:id="R9fe12602599b4eaa"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Decisions" sheetId="7" r:id="R9efafd78e8d84540"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Missing" sheetId="8" r:id="R6efadb3a18804f8a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Current Status" sheetId="1" r:id="Ra50cc49afc9246f4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Datasets" sheetId="2" r:id="Rf9c2af42f71045bf"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Code" sheetId="3" r:id="R44bb86ae8ecc4866"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tables" sheetId="4" r:id="R51b5a7cea5424773"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Figures" sheetId="5" r:id="R71b3bbaf04284e50"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Runs" sheetId="6" r:id="R106a85992d794a49"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Decisions" sheetId="7" r:id="Rcd338fc8d7f14121"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Missing" sheetId="8" r:id="R2c2f6656f96f4ebc"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -476,7 +476,7 @@
     </x:row>
     <x:row r="3" ht="30" customHeight="1">
       <x:c r="A3" s="10" t="str">
-        <x:v>Source: Control Center and registries; generated 2026-09-24T04:01:07+00:00.</x:v>
+        <x:v>Source: Control Center and registries; generated 2026-09-24T04:10:09+00:00.</x:v>
       </x:c>
       <x:c r="B3" s="10"/>
       <x:c r="C3" s="10"/>
@@ -616,7 +616,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R55af4e2bc5c7472d"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rccdcc77c12a2494e"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1608,7 +1608,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5854e4fa98a24fc3"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Red960c7a06e74cb7"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2575,7 +2575,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R57f02e9cb0874f6f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0e4285f6883b47e1"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2958,7 +2958,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0a6c9a80c41946bd"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R893da9a4d97c4539"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3341,7 +3341,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8376aee543384f36"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb21972324c244640"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3604,7 +3604,7 @@
         <x:v>2026-09-24</x:v>
       </x:c>
       <x:c r="C11" s="19" t="str">
-        <x:v>not committed yet</x:v>
+        <x:v>1398a27798b6d690d6a8b9091472de1fbf8a7691</x:v>
       </x:c>
       <x:c r="D11" s="19" t="str">
         <x:v>94d52af2f33639cc336a6967d3fecfdccc2a2fc3f8b6ae265d116ae457ce0f76</x:v>
@@ -3622,7 +3622,7 @@
         <x:v>由verification_report.json记录</x:v>
       </x:c>
       <x:c r="I11" s="19" t="str">
-        <x:v>pending</x:v>
+        <x:v>yes</x:v>
       </x:c>
       <x:c r="J11" s="19" t="str">
         <x:v>双通道同步与研究说明系统</x:v>
@@ -3636,7 +3636,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R98255c7df46c41c6"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re885ca5749e14446"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3959,7 +3959,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1eccc649dca840d6"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb262ad79e5684538"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4076,7 +4076,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8708cd0cb9274156"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re72bbebe804e4c02"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
docs: record public GitHub publication decision
</commit_message>
<xml_diff>
--- a/docs/Research_Project_Map.xlsx
+++ b/docs/Research_Project_Map.xlsx
@@ -2,14 +2,14 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Current Status" sheetId="1" r:id="Ra50cc49afc9246f4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Datasets" sheetId="2" r:id="Rf9c2af42f71045bf"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Code" sheetId="3" r:id="R44bb86ae8ecc4866"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tables" sheetId="4" r:id="R51b5a7cea5424773"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Figures" sheetId="5" r:id="R71b3bbaf04284e50"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Runs" sheetId="6" r:id="R106a85992d794a49"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Decisions" sheetId="7" r:id="Rcd338fc8d7f14121"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Missing" sheetId="8" r:id="R2c2f6656f96f4ebc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Current Status" sheetId="1" r:id="R2372d1d014c04f3b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Datasets" sheetId="2" r:id="R87382723ce4f4176"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Code" sheetId="3" r:id="Rd0deab60e8e1490f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tables" sheetId="4" r:id="R49437b1a6bf14f65"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Figures" sheetId="5" r:id="Rccca5782c30744f0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Runs" sheetId="6" r:id="R4bc8f8bd40ff4234"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Decisions" sheetId="7" r:id="R26d7e203a06440e8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Missing" sheetId="8" r:id="Rcc5c0a95e8424ecf"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -161,7 +161,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="CurrentStatusTable" displayName="CurrentStatusTable" ref="A5:D13" headerRowCount="1">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="CurrentStatusTable" displayName="CurrentStatusTable" ref="A5:D14" headerRowCount="1">
   <x:tableColumns count="4">
     <x:tableColumn id="1" name="分类"/>
     <x:tableColumn id="2" name="项目"/>
@@ -276,7 +276,7 @@
 </file>
 
 <file path=xl/tables/table7.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="7" name="DecisionsTable" displayName="DecisionsTable" ref="A5:H14" headerRowCount="1">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="7" name="DecisionsTable" displayName="DecisionsTable" ref="A5:H15" headerRowCount="1">
   <x:tableColumns count="8">
     <x:tableColumn id="1" name="决策ID"/>
     <x:tableColumn id="2" name="日期"/>
@@ -476,7 +476,7 @@
     </x:row>
     <x:row r="3" ht="30" customHeight="1">
       <x:c r="A3" s="10" t="str">
-        <x:v>Source: Control Center and registries; generated 2026-09-24T04:10:09+00:00.</x:v>
+        <x:v>Source: Control Center and registries; generated 2026-09-24T04:32:35+00:00.</x:v>
       </x:c>
       <x:c r="B3" s="10"/>
       <x:c r="C3" s="10"/>
@@ -543,27 +543,27 @@
         <x:v>Existing Result</x:v>
       </x:c>
       <x:c r="B9" s="19" t="str">
-        <x:v>Interpretation</x:v>
+        <x:v>GitHub publication</x:v>
       </x:c>
       <x:c r="C9" s="19" t="str">
-        <x:v>识别条件相关关系，不识别因果关系</x:v>
+        <x:v>Public repository: yizihao8288-coder/FYP</x:v>
       </x:c>
       <x:c r="D9" s="19" t="str">
-        <x:v>docs/THESIS_EVIDENCE_MATRIX.md</x:v>
+        <x:v>原始行情、处理行情和冻结事件级CSV仍只在DataVault</x:v>
       </x:c>
     </x:row>
     <x:row r="10">
       <x:c r="A10" s="19" t="str">
-        <x:v>Potential Improvement</x:v>
+        <x:v>Existing Result</x:v>
       </x:c>
       <x:c r="B10" s="19" t="str">
-        <x:v>Inference</x:v>
+        <x:v>Interpretation</x:v>
       </x:c>
       <x:c r="C10" s="19" t="str">
-        <x:v>补充stock/date clustered standard errors</x:v>
+        <x:v>识别条件相关关系，不识别因果关系</x:v>
       </x:c>
       <x:c r="D10" s="19" t="str">
-        <x:v>不得替代HC3 baseline</x:v>
+        <x:v>docs/THESIS_EVIDENCE_MATRIX.md</x:v>
       </x:c>
     </x:row>
     <x:row r="11">
@@ -571,40 +571,54 @@
         <x:v>Potential Improvement</x:v>
       </x:c>
       <x:c r="B11" s="19" t="str">
-        <x:v>Controls</x:v>
+        <x:v>Inference</x:v>
       </x:c>
       <x:c r="C11" s="19" t="str">
-        <x:v>年份/市场状态、事件前波动率、历史行业</x:v>
+        <x:v>补充stock/date clustered standard errors</x:v>
       </x:c>
       <x:c r="D11" s="19" t="str">
-        <x:v>新结果必须单独登记</x:v>
+        <x:v>不得替代HC3 baseline</x:v>
       </x:c>
     </x:row>
     <x:row r="12">
       <x:c r="A12" s="19" t="str">
-        <x:v>Recommended Future Work</x:v>
+        <x:v>Potential Improvement</x:v>
       </x:c>
       <x:c r="B12" s="19" t="str">
-        <x:v>Execution design</x:v>
+        <x:v>Controls</x:v>
       </x:c>
       <x:c r="C12" s="19" t="str">
-        <x:v>可构造次日开盘可执行版本</x:v>
+        <x:v>年份/市场状态、事件前波动率、历史行业</x:v>
       </x:c>
       <x:c r="D12" s="19" t="str">
-        <x:v>解决close-based信号的时点问题</x:v>
+        <x:v>新结果必须单独登记</x:v>
       </x:c>
     </x:row>
     <x:row r="13">
       <x:c r="A13" s="19" t="str">
+        <x:v>Recommended Future Work</x:v>
+      </x:c>
+      <x:c r="B13" s="19" t="str">
+        <x:v>Execution design</x:v>
+      </x:c>
+      <x:c r="C13" s="19" t="str">
+        <x:v>可构造次日开盘可执行版本</x:v>
+      </x:c>
+      <x:c r="D13" s="19" t="str">
+        <x:v>解决close-based信号的时点问题</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="14">
+      <x:c r="A14" s="19" t="str">
         <x:v>Open Action</x:v>
       </x:c>
-      <x:c r="B13" s="19" t="str">
+      <x:c r="B14" s="19" t="str">
         <x:v>Off-device backup</x:v>
       </x:c>
-      <x:c r="C13" s="19" t="str">
+      <x:c r="C14" s="19" t="str">
         <x:v>D盘DataVault已建立，私有云尚未接入</x:v>
       </x:c>
-      <x:c r="D13" s="19" t="str">
+      <x:c r="D14" s="19" t="str">
         <x:v>选择同步根目录可位于D盘的客户端</x:v>
       </x:c>
     </x:row>
@@ -616,7 +630,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rccdcc77c12a2494e"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9d737e3c671a4dd4"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1608,7 +1622,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Red960c7a06e74cb7"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R48a0cf529f134ccd"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2575,7 +2589,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0e4285f6883b47e1"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc2472c86a55248ba"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2958,7 +2972,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R893da9a4d97c4539"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re6086b5fdaba495d"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3341,7 +3355,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb21972324c244640"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3bc39911fbb54b3b"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3604,7 +3618,7 @@
         <x:v>2026-09-24</x:v>
       </x:c>
       <x:c r="C11" s="19" t="str">
-        <x:v>1398a27798b6d690d6a8b9091472de1fbf8a7691</x:v>
+        <x:v>c7932e75d2ef7d49efd75c4175987f989ad8f2ce</x:v>
       </x:c>
       <x:c r="D11" s="19" t="str">
         <x:v>94d52af2f33639cc336a6967d3fecfdccc2a2fc3f8b6ae265d116ae457ce0f76</x:v>
@@ -3636,7 +3650,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re885ca5749e14446"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra944f9774e424db9"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3951,6 +3965,32 @@
         <x:v>未来构造次日开盘执行版本</x:v>
       </x:c>
     </x:row>
+    <x:row r="15">
+      <x:c r="A15" s="19" t="str">
+        <x:v>ADR010</x:v>
+      </x:c>
+      <x:c r="B15" s="19" t="str">
+        <x:v>2026-09-24</x:v>
+      </x:c>
+      <x:c r="C15" s="19" t="str">
+        <x:v>GitHub仓库可见性</x:v>
+      </x:c>
+      <x:c r="D15" s="19" t="str">
+        <x:v>private;public</x:v>
+      </x:c>
+      <x:c r="E15" s="19" t="str">
+        <x:v>public by user decision</x:v>
+      </x:c>
+      <x:c r="F15" s="19" t="str">
+        <x:v>用户明确不要求private，希望直接公开管理</x:v>
+      </x:c>
+      <x:c r="G15" s="19" t="str">
+        <x:v>代码、论文结果、hash清单和部分本机路径记录对外可见；原始行情与冻结CSV仍不上传</x:v>
+      </x:c>
+      <x:c r="H15" s="19" t="str">
+        <x:v>答辩或数据许可要求变化时重新评估</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A1:H1"/>
@@ -3959,7 +3999,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb262ad79e5684538"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfbbdba83d1b142a0"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4076,7 +4116,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re72bbebe804e4c02"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3e929d7d1ff047c8"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>